<commit_message>
S3: plantilla corregida (Ke COP, WACC, Criterios), Rf de hoy y precio de equilibrio en slides, lecturas S3 e Interactiva
- plantillas: fórmulas derivadas por nombre de parámetro; textos de Criterios como texto (antes #NAME?)
- slides/s03: Rf 4,20% (ene-2026) vs 4,78% hoy; precio de equilibrio a 12% y a 10,80%
- literatura: Welch 2021 y Drupp et al. (extracto) verificados; bib y revisión actualizados
- interactiva: SEMANA_ACTUAL=4, lecturas S3, asignaciones a05/a06

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plantillas/modelo-financiero-PLANTILLA.xlsx
+++ b/plantillas/modelo-financiero-PLANTILLA.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,6 +51,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="&lt;function B at 0x11fda7d80&gt;"/>
     </font>
     <font>
       <b val="1"/>
@@ -119,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,8 +136,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,12 +147,12 @@
     <xf numFmtId="3" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -796,7 +800,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Precio del producto (USD/t)</t>
         </is>
@@ -806,7 +810,7 @@
       <c r="D5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Rendimiento físico (t/ha)</t>
         </is>
@@ -816,7 +820,7 @@
       <c r="D6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Precio del carbono (USD/t)</t>
         </is>
@@ -826,7 +830,7 @@
       <c r="D7" s="7" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>CapEx de adaptación (USD)</t>
         </is>
@@ -836,27 +840,27 @@
       <c r="D8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>VPN privado</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="23" t="n"/>
-      <c r="D9" s="23" t="n"/>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>VPN social</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="23" t="n"/>
-      <c r="D10" s="23" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>¿Se financia?</t>
         </is>
@@ -1592,52 +1596,52 @@
       <c r="E40" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>— DERIVADOS (no tocar) —</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Ke en USD</t>
         </is>
       </c>
-      <c r="B43" s="12">
+      <c r="B43" s="13">
         <f>B24+B27*B25+B26</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="11" t="inlineStr">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Ke en COP</t>
         </is>
       </c>
-      <c r="B44" s="12">
-        <f>(1+B43)*(1+B29)/(1+B30)-1</f>
+      <c r="B44" s="13">
+        <f>(1+B43)*(1+B30)/(1+B31)-1</f>
         <v/>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="inlineStr">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t>WACC en COP</t>
         </is>
       </c>
-      <c r="B45" s="12">
-        <f>(1-B17)*B44+B17*B18*(1-B19)</f>
+      <c r="B45" s="13">
+        <f>(1-B20)*B44+B20*B21*(1-B22)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>Adicionalidad de carbono</t>
         </is>
       </c>
-      <c r="B46" s="12">
+      <c r="B46" s="13">
         <f>(B37-B38)*44/12*B6</f>
         <v/>
       </c>
@@ -1744,11 +1748,11 @@
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="7" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="n"/>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="13" t="n"/>
+      <c r="E5" s="14" t="n"/>
+      <c r="F5" s="14" t="n"/>
+      <c r="G5" s="14" t="n"/>
+      <c r="H5" s="14" t="n"/>
+      <c r="I5" s="14" t="n"/>
       <c r="J5" s="7" t="n"/>
     </row>
     <row r="6">
@@ -1756,11 +1760,11 @@
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="7" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n"/>
-      <c r="G6" s="13" t="n"/>
-      <c r="H6" s="13" t="n"/>
-      <c r="I6" s="13" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
       <c r="J6" s="7" t="n"/>
     </row>
     <row r="7">
@@ -1768,11 +1772,11 @@
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="7" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
+      <c r="E7" s="14" t="n"/>
+      <c r="F7" s="14" t="n"/>
+      <c r="G7" s="14" t="n"/>
+      <c r="H7" s="14" t="n"/>
+      <c r="I7" s="14" t="n"/>
       <c r="J7" s="7" t="n"/>
     </row>
     <row r="8">
@@ -1780,11 +1784,11 @@
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="7" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n"/>
-      <c r="G8" s="13" t="n"/>
-      <c r="H8" s="13" t="n"/>
-      <c r="I8" s="13" t="n"/>
+      <c r="E8" s="14" t="n"/>
+      <c r="F8" s="14" t="n"/>
+      <c r="G8" s="14" t="n"/>
+      <c r="H8" s="14" t="n"/>
+      <c r="I8" s="14" t="n"/>
       <c r="J8" s="7" t="n"/>
     </row>
     <row r="9">
@@ -1792,11 +1796,11 @@
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="7" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="13" t="n"/>
-      <c r="I9" s="13" t="n"/>
+      <c r="E9" s="14" t="n"/>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="14" t="n"/>
+      <c r="I9" s="14" t="n"/>
       <c r="J9" s="7" t="n"/>
     </row>
     <row r="10">
@@ -1804,11 +1808,11 @@
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="7" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="13" t="n"/>
-      <c r="I10" s="13" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="14" t="n"/>
       <c r="J10" s="7" t="n"/>
     </row>
     <row r="11">
@@ -1816,11 +1820,11 @@
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="7" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="13" t="n"/>
-      <c r="I11" s="13" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="14" t="n"/>
+      <c r="I11" s="14" t="n"/>
       <c r="J11" s="7" t="n"/>
     </row>
     <row r="12">
@@ -1828,11 +1832,11 @@
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="7" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="13" t="n"/>
-      <c r="H12" s="13" t="n"/>
-      <c r="I12" s="13" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
+      <c r="G12" s="14" t="n"/>
+      <c r="H12" s="14" t="n"/>
+      <c r="I12" s="14" t="n"/>
       <c r="J12" s="7" t="n"/>
     </row>
     <row r="13">
@@ -1840,11 +1844,11 @@
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="7" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
-      <c r="I13" s="13" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="14" t="n"/>
+      <c r="I13" s="14" t="n"/>
       <c r="J13" s="7" t="n"/>
     </row>
     <row r="14">
@@ -1852,11 +1856,11 @@
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="7" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
-      <c r="G14" s="13" t="n"/>
-      <c r="H14" s="13" t="n"/>
-      <c r="I14" s="13" t="n"/>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="14" t="n"/>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="14" t="n"/>
+      <c r="I14" s="14" t="n"/>
       <c r="J14" s="7" t="n"/>
     </row>
     <row r="15">
@@ -1864,11 +1868,11 @@
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="7" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
-      <c r="G15" s="13" t="n"/>
-      <c r="H15" s="13" t="n"/>
-      <c r="I15" s="13" t="n"/>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n"/>
+      <c r="G15" s="14" t="n"/>
+      <c r="H15" s="14" t="n"/>
+      <c r="I15" s="14" t="n"/>
       <c r="J15" s="7" t="n"/>
     </row>
     <row r="16">
@@ -1876,11 +1880,11 @@
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="7" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="13" t="n"/>
-      <c r="I16" s="13" t="n"/>
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="14" t="n"/>
       <c r="J16" s="7" t="n"/>
     </row>
     <row r="17">
@@ -1888,11 +1892,11 @@
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="7" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="13" t="n"/>
-      <c r="I17" s="13" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="14" t="n"/>
+      <c r="I17" s="14" t="n"/>
       <c r="J17" s="7" t="n"/>
     </row>
     <row r="18">
@@ -1900,11 +1904,11 @@
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="7" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
-      <c r="G18" s="13" t="n"/>
-      <c r="H18" s="13" t="n"/>
-      <c r="I18" s="13" t="n"/>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="14" t="n"/>
       <c r="J18" s="7" t="n"/>
     </row>
     <row r="19">
@@ -1912,11 +1916,11 @@
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="7" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
-      <c r="G19" s="13" t="n"/>
-      <c r="H19" s="13" t="n"/>
-      <c r="I19" s="13" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="14" t="n"/>
       <c r="J19" s="7" t="n"/>
     </row>
     <row r="20">
@@ -1924,11 +1928,11 @@
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="7" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
-      <c r="G20" s="13" t="n"/>
-      <c r="H20" s="13" t="n"/>
-      <c r="I20" s="13" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="14" t="n"/>
       <c r="J20" s="7" t="n"/>
     </row>
     <row r="21">
@@ -1936,11 +1940,11 @@
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="7" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n"/>
-      <c r="G21" s="13" t="n"/>
-      <c r="H21" s="13" t="n"/>
-      <c r="I21" s="13" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="14" t="n"/>
       <c r="J21" s="7" t="n"/>
     </row>
     <row r="22">
@@ -1948,11 +1952,11 @@
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="7" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="13" t="n"/>
-      <c r="H22" s="13" t="n"/>
-      <c r="I22" s="13" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="14" t="n"/>
       <c r="J22" s="7" t="n"/>
     </row>
     <row r="23">
@@ -1960,11 +1964,11 @@
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="7" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="13" t="n"/>
-      <c r="H23" s="13" t="n"/>
-      <c r="I23" s="13" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="14" t="n"/>
+      <c r="I23" s="14" t="n"/>
       <c r="J23" s="7" t="n"/>
     </row>
     <row r="24">
@@ -1972,15 +1976,15 @@
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="7" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="13" t="n"/>
+      <c r="E24" s="14" t="n"/>
+      <c r="F24" s="14" t="n"/>
+      <c r="G24" s="14" t="n"/>
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="14" t="n"/>
       <c r="J24" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
@@ -2189,76 +2193,76 @@
       <c r="E24" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>OpEx por año (USD/ha) — curva de maduración</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="B29" s="15" t="n">
+      <c r="B29" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="15" t="n">
+      <c r="C29" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D29" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="15" t="n">
+      <c r="E29" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="15" t="n">
+      <c r="F29" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="G29" s="15" t="n">
+      <c r="G29" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="H29" s="15" t="n">
+      <c r="H29" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="I29" s="15" t="n">
+      <c r="I29" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="J29" s="15" t="n">
+      <c r="J29" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="K29" s="15" t="n">
+      <c r="K29" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="L29" s="15" t="n">
+      <c r="L29" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="M29" s="15" t="n">
+      <c r="M29" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="N29" s="15" t="n">
+      <c r="N29" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="O29" s="15" t="n">
+      <c r="O29" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="P29" s="15" t="n">
+      <c r="P29" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="Q29" s="15" t="n">
+      <c r="Q29" s="16" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>OpEx USD/ha</t>
         </is>
@@ -2312,159 +2316,159 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n"/>
-      <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="15" t="n">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="15" t="n">
+      <c r="L4" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="M4" s="15" t="n">
+      <c r="M4" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="N4" s="15" t="n">
+      <c r="N4" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="O4" s="15" t="n">
+      <c r="O4" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="P4" s="15" t="n">
+      <c r="P4" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="Q4" s="15" t="n">
+      <c r="Q4" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="R4" s="15" t="n">
+      <c r="R4" s="16" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Ingresos operativos</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
-      <c r="N5" s="16" t="n"/>
-      <c r="O5" s="16" t="n"/>
-      <c r="P5" s="16" t="n"/>
-      <c r="Q5" s="16" t="n"/>
-      <c r="R5" s="16" t="n"/>
+      <c r="C5" s="17" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="17" t="n"/>
+      <c r="O5" s="17" t="n"/>
+      <c r="P5" s="17" t="n"/>
+      <c r="Q5" s="17" t="n"/>
+      <c r="R5" s="17" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Costos operativos</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="16" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="16" t="n"/>
-      <c r="N6" s="16" t="n"/>
-      <c r="O6" s="16" t="n"/>
-      <c r="P6" s="16" t="n"/>
-      <c r="Q6" s="16" t="n"/>
-      <c r="R6" s="16" t="n"/>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="17" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="17" t="n"/>
+      <c r="M6" s="17" t="n"/>
+      <c r="N6" s="17" t="n"/>
+      <c r="O6" s="17" t="n"/>
+      <c r="P6" s="17" t="n"/>
+      <c r="Q6" s="17" t="n"/>
+      <c r="R6" s="17" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Flujo operativo</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
+      <c r="R7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>ACUMULADO</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="18" t="n"/>
-      <c r="G8" s="18" t="n"/>
-      <c r="H8" s="18" t="n"/>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="18" t="n"/>
-      <c r="N8" s="18" t="n"/>
-      <c r="O8" s="18" t="n"/>
-      <c r="P8" s="18" t="n"/>
-      <c r="Q8" s="18" t="n"/>
-      <c r="R8" s="18" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="19" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="19" t="n"/>
+      <c r="P8" s="19" t="n"/>
+      <c r="Q8" s="19" t="n"/>
+      <c r="R8" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>DÉFICIT ACUMULADO MÁXIMO =</t>
         </is>
       </c>
-      <c r="D10" s="19" t="n"/>
+      <c r="D10" s="20" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>→ Se invierte en año 0 y SE RECUPERA en año 15</t>
         </is>
@@ -2502,54 +2506,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n"/>
-      <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="15" t="n">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="15" t="n">
+      <c r="L4" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="M4" s="15" t="n">
+      <c r="M4" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="N4" s="15" t="n">
+      <c r="N4" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="O4" s="15" t="n">
+      <c r="O4" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="P4" s="15" t="n">
+      <c r="P4" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="Q4" s="15" t="n">
+      <c r="Q4" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="R4" s="15" t="n">
+      <c r="R4" s="16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2559,22 +2563,22 @@
           <t>Ingresos</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
+      <c r="R5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -2582,22 +2586,22 @@
           <t>(−) Costos operativos</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n"/>
-      <c r="O6" s="17" t="n"/>
-      <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="18" t="n"/>
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="18" t="n"/>
+      <c r="O6" s="18" t="n"/>
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="n"/>
+      <c r="R6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -2605,45 +2609,45 @@
           <t>(−) Depreciación</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
+      <c r="R7" s="18" t="n"/>
     </row>
     <row r="8">
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>(=) EBIT</t>
         </is>
       </c>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
-      <c r="E8" s="21" t="n"/>
-      <c r="F8" s="21" t="n"/>
-      <c r="G8" s="21" t="n"/>
-      <c r="H8" s="21" t="n"/>
-      <c r="I8" s="21" t="n"/>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="21" t="n"/>
-      <c r="L8" s="21" t="n"/>
-      <c r="M8" s="21" t="n"/>
-      <c r="N8" s="21" t="n"/>
-      <c r="O8" s="21" t="n"/>
-      <c r="P8" s="21" t="n"/>
-      <c r="Q8" s="21" t="n"/>
-      <c r="R8" s="21" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="22" t="n"/>
+      <c r="H8" s="22" t="n"/>
+      <c r="I8" s="22" t="n"/>
+      <c r="J8" s="22" t="n"/>
+      <c r="K8" s="22" t="n"/>
+      <c r="L8" s="22" t="n"/>
+      <c r="M8" s="22" t="n"/>
+      <c r="N8" s="22" t="n"/>
+      <c r="O8" s="22" t="n"/>
+      <c r="P8" s="22" t="n"/>
+      <c r="Q8" s="22" t="n"/>
+      <c r="R8" s="22" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
@@ -2651,22 +2655,22 @@
           <t>(−) Impuestos  ⚠ CERO si EBIT&lt;0</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="17" t="n"/>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="17" t="n"/>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="17" t="n"/>
-      <c r="N9" s="17" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="17" t="n"/>
-      <c r="Q9" s="17" t="n"/>
-      <c r="R9" s="17" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="18" t="n"/>
+      <c r="O9" s="18" t="n"/>
+      <c r="P9" s="18" t="n"/>
+      <c r="Q9" s="18" t="n"/>
+      <c r="R9" s="18" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
@@ -2674,22 +2678,22 @@
           <t>(+) Depreciación</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="17" t="n"/>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="17" t="n"/>
-      <c r="R10" s="17" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n"/>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="18" t="n"/>
+      <c r="L10" s="18" t="n"/>
+      <c r="M10" s="18" t="n"/>
+      <c r="N10" s="18" t="n"/>
+      <c r="O10" s="18" t="n"/>
+      <c r="P10" s="18" t="n"/>
+      <c r="Q10" s="18" t="n"/>
+      <c r="R10" s="18" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="3" t="inlineStr">
@@ -2697,22 +2701,22 @@
           <t>(−) CapEx</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n"/>
-      <c r="D11" s="17" t="n"/>
-      <c r="E11" s="17" t="n"/>
-      <c r="F11" s="17" t="n"/>
-      <c r="G11" s="17" t="n"/>
-      <c r="H11" s="17" t="n"/>
-      <c r="I11" s="17" t="n"/>
-      <c r="J11" s="17" t="n"/>
-      <c r="K11" s="17" t="n"/>
-      <c r="L11" s="17" t="n"/>
-      <c r="M11" s="17" t="n"/>
-      <c r="N11" s="17" t="n"/>
-      <c r="O11" s="17" t="n"/>
-      <c r="P11" s="17" t="n"/>
-      <c r="Q11" s="17" t="n"/>
-      <c r="R11" s="17" t="n"/>
+      <c r="C11" s="18" t="n"/>
+      <c r="D11" s="18" t="n"/>
+      <c r="E11" s="18" t="n"/>
+      <c r="F11" s="18" t="n"/>
+      <c r="G11" s="18" t="n"/>
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="18" t="n"/>
+      <c r="J11" s="18" t="n"/>
+      <c r="K11" s="18" t="n"/>
+      <c r="L11" s="18" t="n"/>
+      <c r="M11" s="18" t="n"/>
+      <c r="N11" s="18" t="n"/>
+      <c r="O11" s="18" t="n"/>
+      <c r="P11" s="18" t="n"/>
+      <c r="Q11" s="18" t="n"/>
+      <c r="R11" s="18" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
@@ -2720,22 +2724,22 @@
           <t>(−) Δ Capital de trabajo</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="n"/>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="17" t="n"/>
-      <c r="M12" s="17" t="n"/>
-      <c r="N12" s="17" t="n"/>
-      <c r="O12" s="17" t="n"/>
-      <c r="P12" s="17" t="n"/>
-      <c r="Q12" s="17" t="n"/>
-      <c r="R12" s="17" t="n"/>
+      <c r="C12" s="18" t="n"/>
+      <c r="D12" s="18" t="n"/>
+      <c r="E12" s="18" t="n"/>
+      <c r="F12" s="18" t="n"/>
+      <c r="G12" s="18" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="18" t="n"/>
+      <c r="J12" s="18" t="n"/>
+      <c r="K12" s="18" t="n"/>
+      <c r="L12" s="18" t="n"/>
+      <c r="M12" s="18" t="n"/>
+      <c r="N12" s="18" t="n"/>
+      <c r="O12" s="18" t="n"/>
+      <c r="P12" s="18" t="n"/>
+      <c r="Q12" s="18" t="n"/>
+      <c r="R12" s="18" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
@@ -2743,45 +2747,45 @@
           <t>(+) Valor terminal</t>
         </is>
       </c>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="17" t="n"/>
-      <c r="G13" s="17" t="n"/>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="17" t="n"/>
-      <c r="K13" s="17" t="n"/>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="17" t="n"/>
-      <c r="O13" s="17" t="n"/>
-      <c r="P13" s="17" t="n"/>
-      <c r="Q13" s="17" t="n"/>
-      <c r="R13" s="17" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="18" t="n"/>
+      <c r="M13" s="18" t="n"/>
+      <c r="N13" s="18" t="n"/>
+      <c r="O13" s="18" t="n"/>
+      <c r="P13" s="18" t="n"/>
+      <c r="Q13" s="18" t="n"/>
+      <c r="R13" s="18" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>(=) FCLD</t>
         </is>
       </c>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
-      <c r="E14" s="21" t="n"/>
-      <c r="F14" s="21" t="n"/>
-      <c r="G14" s="21" t="n"/>
-      <c r="H14" s="21" t="n"/>
-      <c r="I14" s="21" t="n"/>
-      <c r="J14" s="21" t="n"/>
-      <c r="K14" s="21" t="n"/>
-      <c r="L14" s="21" t="n"/>
-      <c r="M14" s="21" t="n"/>
-      <c r="N14" s="21" t="n"/>
-      <c r="O14" s="21" t="n"/>
-      <c r="P14" s="21" t="n"/>
-      <c r="Q14" s="21" t="n"/>
-      <c r="R14" s="21" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+      <c r="G14" s="22" t="n"/>
+      <c r="H14" s="22" t="n"/>
+      <c r="I14" s="22" t="n"/>
+      <c r="J14" s="22" t="n"/>
+      <c r="K14" s="22" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="22" t="n"/>
+      <c r="N14" s="22" t="n"/>
+      <c r="O14" s="22" t="n"/>
+      <c r="P14" s="22" t="n"/>
+      <c r="Q14" s="22" t="n"/>
+      <c r="R14" s="22" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2815,54 +2819,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n"/>
-      <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="15" t="n">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="15" t="n">
+      <c r="L4" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="M4" s="15" t="n">
+      <c r="M4" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="N4" s="15" t="n">
+      <c r="N4" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="O4" s="15" t="n">
+      <c r="O4" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="P4" s="15" t="n">
+      <c r="P4" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="Q4" s="15" t="n">
+      <c r="Q4" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="R4" s="15" t="n">
+      <c r="R4" s="16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2872,22 +2876,22 @@
           <t>FCLD</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
+      <c r="R5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -2895,22 +2899,22 @@
           <t>(+) Desembolso de deuda</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n"/>
-      <c r="O6" s="17" t="n"/>
-      <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="18" t="n"/>
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="18" t="n"/>
+      <c r="O6" s="18" t="n"/>
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="n"/>
+      <c r="R6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -2918,22 +2922,22 @@
           <t>(−) Intereses × (1−t)</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
+      <c r="R7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
@@ -2941,102 +2945,102 @@
           <t>(−) Amortización de capital</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="17" t="n"/>
-      <c r="K8" s="17" t="n"/>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="17" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="17" t="n"/>
-      <c r="Q8" s="17" t="n"/>
-      <c r="R8" s="17" t="n"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="18" t="n"/>
+      <c r="O8" s="18" t="n"/>
+      <c r="P8" s="18" t="n"/>
+      <c r="Q8" s="18" t="n"/>
+      <c r="R8" s="18" t="n"/>
     </row>
     <row r="9">
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>(=) FCA</t>
         </is>
       </c>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
-      <c r="E9" s="21" t="n"/>
-      <c r="F9" s="21" t="n"/>
-      <c r="G9" s="21" t="n"/>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="21" t="n"/>
-      <c r="J9" s="21" t="n"/>
-      <c r="K9" s="21" t="n"/>
-      <c r="L9" s="21" t="n"/>
-      <c r="M9" s="21" t="n"/>
-      <c r="N9" s="21" t="n"/>
-      <c r="O9" s="21" t="n"/>
-      <c r="P9" s="21" t="n"/>
-      <c r="Q9" s="21" t="n"/>
-      <c r="R9" s="21" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="22" t="n"/>
+      <c r="I9" s="22" t="n"/>
+      <c r="J9" s="22" t="n"/>
+      <c r="K9" s="22" t="n"/>
+      <c r="L9" s="22" t="n"/>
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="22" t="n"/>
+      <c r="O9" s="22" t="n"/>
+      <c r="P9" s="22" t="n"/>
+      <c r="Q9" s="22" t="n"/>
+      <c r="R9" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>TABLA DE AMORTIZACIÓN</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="15" t="n">
+      <c r="A12" s="14" t="n"/>
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H12" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I12" s="15" t="n">
+      <c r="I12" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J12" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="K12" s="15" t="n">
+      <c r="K12" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="L12" s="15" t="n">
+      <c r="L12" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="M12" s="15" t="n">
+      <c r="M12" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="N12" s="15" t="n">
+      <c r="N12" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="O12" s="15" t="n">
+      <c r="O12" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="P12" s="15" t="n">
+      <c r="P12" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="Q12" s="15" t="n">
+      <c r="Q12" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="R12" s="15" t="n">
+      <c r="R12" s="16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3046,22 +3050,22 @@
           <t>Saldo inicial</t>
         </is>
       </c>
-      <c r="C13" s="17" t="n"/>
-      <c r="D13" s="17" t="n"/>
-      <c r="E13" s="17" t="n"/>
-      <c r="F13" s="17" t="n"/>
-      <c r="G13" s="17" t="n"/>
-      <c r="H13" s="17" t="n"/>
-      <c r="I13" s="17" t="n"/>
-      <c r="J13" s="17" t="n"/>
-      <c r="K13" s="17" t="n"/>
-      <c r="L13" s="17" t="n"/>
-      <c r="M13" s="17" t="n"/>
-      <c r="N13" s="17" t="n"/>
-      <c r="O13" s="17" t="n"/>
-      <c r="P13" s="17" t="n"/>
-      <c r="Q13" s="17" t="n"/>
-      <c r="R13" s="17" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="18" t="n"/>
+      <c r="J13" s="18" t="n"/>
+      <c r="K13" s="18" t="n"/>
+      <c r="L13" s="18" t="n"/>
+      <c r="M13" s="18" t="n"/>
+      <c r="N13" s="18" t="n"/>
+      <c r="O13" s="18" t="n"/>
+      <c r="P13" s="18" t="n"/>
+      <c r="Q13" s="18" t="n"/>
+      <c r="R13" s="18" t="n"/>
     </row>
     <row r="14">
       <c r="B14" t="inlineStr">
@@ -3069,22 +3073,22 @@
           <t>Intereses</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="17" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n"/>
-      <c r="I14" s="17" t="n"/>
-      <c r="J14" s="17" t="n"/>
-      <c r="K14" s="17" t="n"/>
-      <c r="L14" s="17" t="n"/>
-      <c r="M14" s="17" t="n"/>
-      <c r="N14" s="17" t="n"/>
-      <c r="O14" s="17" t="n"/>
-      <c r="P14" s="17" t="n"/>
-      <c r="Q14" s="17" t="n"/>
-      <c r="R14" s="17" t="n"/>
+      <c r="C14" s="18" t="n"/>
+      <c r="D14" s="18" t="n"/>
+      <c r="E14" s="18" t="n"/>
+      <c r="F14" s="18" t="n"/>
+      <c r="G14" s="18" t="n"/>
+      <c r="H14" s="18" t="n"/>
+      <c r="I14" s="18" t="n"/>
+      <c r="J14" s="18" t="n"/>
+      <c r="K14" s="18" t="n"/>
+      <c r="L14" s="18" t="n"/>
+      <c r="M14" s="18" t="n"/>
+      <c r="N14" s="18" t="n"/>
+      <c r="O14" s="18" t="n"/>
+      <c r="P14" s="18" t="n"/>
+      <c r="Q14" s="18" t="n"/>
+      <c r="R14" s="18" t="n"/>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
@@ -3092,22 +3096,22 @@
           <t>Amortización</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="17" t="n"/>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="17" t="n"/>
-      <c r="H15" s="17" t="n"/>
-      <c r="I15" s="17" t="n"/>
-      <c r="J15" s="17" t="n"/>
-      <c r="K15" s="17" t="n"/>
-      <c r="L15" s="17" t="n"/>
-      <c r="M15" s="17" t="n"/>
-      <c r="N15" s="17" t="n"/>
-      <c r="O15" s="17" t="n"/>
-      <c r="P15" s="17" t="n"/>
-      <c r="Q15" s="17" t="n"/>
-      <c r="R15" s="17" t="n"/>
+      <c r="C15" s="18" t="n"/>
+      <c r="D15" s="18" t="n"/>
+      <c r="E15" s="18" t="n"/>
+      <c r="F15" s="18" t="n"/>
+      <c r="G15" s="18" t="n"/>
+      <c r="H15" s="18" t="n"/>
+      <c r="I15" s="18" t="n"/>
+      <c r="J15" s="18" t="n"/>
+      <c r="K15" s="18" t="n"/>
+      <c r="L15" s="18" t="n"/>
+      <c r="M15" s="18" t="n"/>
+      <c r="N15" s="18" t="n"/>
+      <c r="O15" s="18" t="n"/>
+      <c r="P15" s="18" t="n"/>
+      <c r="Q15" s="18" t="n"/>
+      <c r="R15" s="18" t="n"/>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
@@ -3115,22 +3119,22 @@
           <t>Saldo final</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="17" t="n"/>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="17" t="n"/>
-      <c r="I16" s="17" t="n"/>
-      <c r="J16" s="17" t="n"/>
-      <c r="K16" s="17" t="n"/>
-      <c r="L16" s="17" t="n"/>
-      <c r="M16" s="17" t="n"/>
-      <c r="N16" s="17" t="n"/>
-      <c r="O16" s="17" t="n"/>
-      <c r="P16" s="17" t="n"/>
-      <c r="Q16" s="17" t="n"/>
-      <c r="R16" s="17" t="n"/>
+      <c r="C16" s="18" t="n"/>
+      <c r="D16" s="18" t="n"/>
+      <c r="E16" s="18" t="n"/>
+      <c r="F16" s="18" t="n"/>
+      <c r="G16" s="18" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="18" t="n"/>
+      <c r="J16" s="18" t="n"/>
+      <c r="K16" s="18" t="n"/>
+      <c r="L16" s="18" t="n"/>
+      <c r="M16" s="18" t="n"/>
+      <c r="N16" s="18" t="n"/>
+      <c r="O16" s="18" t="n"/>
+      <c r="P16" s="18" t="n"/>
+      <c r="Q16" s="18" t="n"/>
+      <c r="R16" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3195,255 +3199,262 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>VPN del proyecto @ WACC</t>
         </is>
       </c>
-      <c r="B5" s="23" t="n"/>
-      <c r="C5" s="13">
-        <f>VNA(WACC; F1:F15)+F0</f>
-        <v/>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>=VNA(WACC; F1:F15)+F0</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Crea o destruye valor</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr"/>
+      <c r="E5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>VPN @ WACC límite inferior</t>
         </is>
       </c>
-      <c r="B6" s="23" t="n"/>
-      <c r="C6" s="13" t="inlineStr"/>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="B6" s="24" t="n"/>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr">
         <is>
           <t>Robustez</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>VPN @ WACC límite superior</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n"/>
-      <c r="C7" s="13" t="inlineStr"/>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="B7" s="24" t="n"/>
+      <c r="C7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Robustez</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr"/>
+      <c r="E7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>VPN del accionista @ Ke</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n"/>
-      <c r="C8" s="13">
-        <f>VNA(Ke; ...)+F0</f>
-        <v/>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="B8" s="24" t="n"/>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>=VNA(Ke; ...)+F0</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Retorno al patrimonio</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>≠ VPN del proyecto</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>TIR</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
-      <c r="C9" s="13">
-        <f>TIR(rango)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>=TIR(rango)</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Eficiencia</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>⚠ verificar signos</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>TIR Modificada</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n"/>
-      <c r="C10" s="13">
-        <f>TIRM(rango; Kd; WACC)</f>
-        <v/>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>=TIRM(rango; Kd; WACC)</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
         <is>
           <t>Eficiencia honesta</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Siempre única</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>Payback descontado</t>
         </is>
       </c>
-      <c r="B11" s="23" t="n"/>
-      <c r="C11" s="13" t="inlineStr"/>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="14" t="inlineStr"/>
+      <c r="D11" s="14" t="inlineStr">
         <is>
           <t>Exposición temporal</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr"/>
+      <c r="E11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>Costo Anual Equivalente</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="13">
-        <f>PAGO(WACC; n; -VPN)</f>
-        <v/>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>=PAGO(WACC; n; -VPN)</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
         <is>
           <t>Comparar vidas distintas</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Índice de rentabilidad</t>
         </is>
       </c>
-      <c r="B13" s="23" t="n"/>
-      <c r="C13" s="13">
-        <f>VPN/Inversión</f>
-        <v/>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>=VPN/Inversión</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
         <is>
           <t>Racionamiento de capital</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Precio de equilibrio</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n"/>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Buscar objetivo</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="D14" s="14" t="inlineStr">
         <is>
           <t>¿A qué precio VPN=0?</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>LA cifra comunicable</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Punto de equilibrio (t)</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n"/>
-      <c r="C15" s="13">
-        <f>CF/(p−cv)</f>
-        <v/>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>=CF/(p−cv)</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
         <is>
           <t>Volumen mínimo</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr"/>
+      <c r="E15" s="14" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>GAO</t>
         </is>
       </c>
-      <c r="B16" s="23" t="n"/>
-      <c r="C16" s="13" t="inlineStr"/>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="B16" s="24" t="n"/>
+      <c r="C16" s="14" t="inlineStr"/>
+      <c r="D16" s="14" t="inlineStr">
         <is>
           <t>Sensibilidad operativa</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr"/>
+      <c r="E16" s="14" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>GAF</t>
         </is>
       </c>
-      <c r="B17" s="23" t="n"/>
-      <c r="C17" s="13" t="inlineStr"/>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="14" t="inlineStr"/>
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>Sensibilidad financiera</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr"/>
+      <c r="E17" s="14" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Cambios de signo del flujo</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="13" t="inlineStr"/>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="14" t="inlineStr"/>
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t>¿TIR confiable?</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="14" t="inlineStr">
         <is>
           <t>⚠ si &gt;1, declararlo</t>
         </is>
@@ -3481,54 +3492,54 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n"/>
-      <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="15" t="n">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="15" t="inlineStr"/>
+      <c r="C4" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="15" t="n">
+      <c r="L4" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="M4" s="15" t="n">
+      <c r="M4" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="N4" s="15" t="n">
+      <c r="N4" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="O4" s="15" t="n">
+      <c r="O4" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="P4" s="15" t="n">
+      <c r="P4" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="Q4" s="15" t="n">
+      <c r="Q4" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="R4" s="15" t="n">
+      <c r="R4" s="16" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3538,22 +3549,22 @@
           <t>FCLD privado</t>
         </is>
       </c>
-      <c r="C5" s="17" t="n"/>
-      <c r="D5" s="17" t="n"/>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="17" t="n"/>
-      <c r="G5" s="17" t="n"/>
-      <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
-      <c r="J5" s="17" t="n"/>
-      <c r="K5" s="17" t="n"/>
-      <c r="L5" s="17" t="n"/>
-      <c r="M5" s="17" t="n"/>
-      <c r="N5" s="17" t="n"/>
-      <c r="O5" s="17" t="n"/>
-      <c r="P5" s="17" t="n"/>
-      <c r="Q5" s="17" t="n"/>
-      <c r="R5" s="17" t="n"/>
+      <c r="C5" s="18" t="n"/>
+      <c r="D5" s="18" t="n"/>
+      <c r="E5" s="18" t="n"/>
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="18" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="18" t="n"/>
+      <c r="J5" s="18" t="n"/>
+      <c r="K5" s="18" t="n"/>
+      <c r="L5" s="18" t="n"/>
+      <c r="M5" s="18" t="n"/>
+      <c r="N5" s="18" t="n"/>
+      <c r="O5" s="18" t="n"/>
+      <c r="P5" s="18" t="n"/>
+      <c r="Q5" s="18" t="n"/>
+      <c r="R5" s="18" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
@@ -3561,22 +3572,22 @@
           <t>(−) Eliminar impuestos  [transferencia]</t>
         </is>
       </c>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="17" t="n"/>
-      <c r="J6" s="17" t="n"/>
-      <c r="K6" s="17" t="n"/>
-      <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
-      <c r="N6" s="17" t="n"/>
-      <c r="O6" s="17" t="n"/>
-      <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="18" t="n"/>
+      <c r="J6" s="18" t="n"/>
+      <c r="K6" s="18" t="n"/>
+      <c r="L6" s="18" t="n"/>
+      <c r="M6" s="18" t="n"/>
+      <c r="N6" s="18" t="n"/>
+      <c r="O6" s="18" t="n"/>
+      <c r="P6" s="18" t="n"/>
+      <c r="Q6" s="18" t="n"/>
+      <c r="R6" s="18" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="inlineStr">
@@ -3584,22 +3595,22 @@
           <t>(−) Eliminar prima de certificación  [transferencia]</t>
         </is>
       </c>
-      <c r="C7" s="17" t="n"/>
-      <c r="D7" s="17" t="n"/>
-      <c r="E7" s="17" t="n"/>
-      <c r="F7" s="17" t="n"/>
-      <c r="G7" s="17" t="n"/>
-      <c r="H7" s="17" t="n"/>
-      <c r="I7" s="17" t="n"/>
-      <c r="J7" s="17" t="n"/>
-      <c r="K7" s="17" t="n"/>
-      <c r="L7" s="17" t="n"/>
-      <c r="M7" s="17" t="n"/>
-      <c r="N7" s="17" t="n"/>
-      <c r="O7" s="17" t="n"/>
-      <c r="P7" s="17" t="n"/>
-      <c r="Q7" s="17" t="n"/>
-      <c r="R7" s="17" t="n"/>
+      <c r="C7" s="18" t="n"/>
+      <c r="D7" s="18" t="n"/>
+      <c r="E7" s="18" t="n"/>
+      <c r="F7" s="18" t="n"/>
+      <c r="G7" s="18" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="18" t="n"/>
+      <c r="J7" s="18" t="n"/>
+      <c r="K7" s="18" t="n"/>
+      <c r="L7" s="18" t="n"/>
+      <c r="M7" s="18" t="n"/>
+      <c r="N7" s="18" t="n"/>
+      <c r="O7" s="18" t="n"/>
+      <c r="P7" s="18" t="n"/>
+      <c r="Q7" s="18" t="n"/>
+      <c r="R7" s="18" t="n"/>
     </row>
     <row r="8">
       <c r="B8" s="3" t="inlineStr">
@@ -3607,22 +3618,22 @@
           <t>(±) Ajuste por salario sombra</t>
         </is>
       </c>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="17" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="17" t="n"/>
-      <c r="J8" s="17" t="n"/>
-      <c r="K8" s="17" t="n"/>
-      <c r="L8" s="17" t="n"/>
-      <c r="M8" s="17" t="n"/>
-      <c r="N8" s="17" t="n"/>
-      <c r="O8" s="17" t="n"/>
-      <c r="P8" s="17" t="n"/>
-      <c r="Q8" s="17" t="n"/>
-      <c r="R8" s="17" t="n"/>
+      <c r="C8" s="18" t="n"/>
+      <c r="D8" s="18" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="18" t="n"/>
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="18" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="18" t="n"/>
+      <c r="M8" s="18" t="n"/>
+      <c r="N8" s="18" t="n"/>
+      <c r="O8" s="18" t="n"/>
+      <c r="P8" s="18" t="n"/>
+      <c r="Q8" s="18" t="n"/>
+      <c r="R8" s="18" t="n"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="inlineStr">
@@ -3630,22 +3641,22 @@
           <t>(+) Carbono removido × precio sombra</t>
         </is>
       </c>
-      <c r="C9" s="17" t="n"/>
-      <c r="D9" s="17" t="n"/>
-      <c r="E9" s="17" t="n"/>
-      <c r="F9" s="17" t="n"/>
-      <c r="G9" s="17" t="n"/>
-      <c r="H9" s="17" t="n"/>
-      <c r="I9" s="17" t="n"/>
-      <c r="J9" s="17" t="n"/>
-      <c r="K9" s="17" t="n"/>
-      <c r="L9" s="17" t="n"/>
-      <c r="M9" s="17" t="n"/>
-      <c r="N9" s="17" t="n"/>
-      <c r="O9" s="17" t="n"/>
-      <c r="P9" s="17" t="n"/>
-      <c r="Q9" s="17" t="n"/>
-      <c r="R9" s="17" t="n"/>
+      <c r="C9" s="18" t="n"/>
+      <c r="D9" s="18" t="n"/>
+      <c r="E9" s="18" t="n"/>
+      <c r="F9" s="18" t="n"/>
+      <c r="G9" s="18" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="18" t="n"/>
+      <c r="J9" s="18" t="n"/>
+      <c r="K9" s="18" t="n"/>
+      <c r="L9" s="18" t="n"/>
+      <c r="M9" s="18" t="n"/>
+      <c r="N9" s="18" t="n"/>
+      <c r="O9" s="18" t="n"/>
+      <c r="P9" s="18" t="n"/>
+      <c r="Q9" s="18" t="n"/>
+      <c r="R9" s="18" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
@@ -3653,48 +3664,48 @@
           <t>(+) Otra externalidad (agua / biodiversidad)</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="17" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="17" t="n"/>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="17" t="n"/>
-      <c r="J10" s="17" t="n"/>
-      <c r="K10" s="17" t="n"/>
-      <c r="L10" s="17" t="n"/>
-      <c r="M10" s="17" t="n"/>
-      <c r="N10" s="17" t="n"/>
-      <c r="O10" s="17" t="n"/>
-      <c r="P10" s="17" t="n"/>
-      <c r="Q10" s="17" t="n"/>
-      <c r="R10" s="17" t="n"/>
+      <c r="C10" s="18" t="n"/>
+      <c r="D10" s="18" t="n"/>
+      <c r="E10" s="18" t="n"/>
+      <c r="F10" s="18" t="n"/>
+      <c r="G10" s="18" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="18" t="n"/>
+      <c r="K10" s="18" t="n"/>
+      <c r="L10" s="18" t="n"/>
+      <c r="M10" s="18" t="n"/>
+      <c r="N10" s="18" t="n"/>
+      <c r="O10" s="18" t="n"/>
+      <c r="P10" s="18" t="n"/>
+      <c r="Q10" s="18" t="n"/>
+      <c r="R10" s="18" t="n"/>
     </row>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>(=) FLUJO SOCIAL</t>
         </is>
       </c>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="21" t="n"/>
-      <c r="G11" s="21" t="n"/>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="21" t="n"/>
-      <c r="J11" s="21" t="n"/>
-      <c r="K11" s="21" t="n"/>
-      <c r="L11" s="21" t="n"/>
-      <c r="M11" s="21" t="n"/>
-      <c r="N11" s="21" t="n"/>
-      <c r="O11" s="21" t="n"/>
-      <c r="P11" s="21" t="n"/>
-      <c r="Q11" s="21" t="n"/>
-      <c r="R11" s="21" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+      <c r="G11" s="22" t="n"/>
+      <c r="H11" s="22" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="22" t="n"/>
+      <c r="K11" s="22" t="n"/>
+      <c r="L11" s="22" t="n"/>
+      <c r="M11" s="22" t="n"/>
+      <c r="N11" s="22" t="n"/>
+      <c r="O11" s="22" t="n"/>
+      <c r="P11" s="22" t="n"/>
+      <c r="Q11" s="22" t="n"/>
+      <c r="R11" s="22" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>PROTOCOLO BANCO MUNDIAL</t>
         </is>
@@ -3728,9 +3739,9 @@
           <t>TSD ambiental Colombia (Res. 1092/2022)</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
-      <c r="E16" s="18" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
@@ -3738,9 +3749,9 @@
           <t>TSD general 9,0%</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
-      <c r="E17" s="18" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -3748,9 +3759,9 @@
           <t>Consenso experto internacional 2,0%</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
-      <c r="E18" s="18" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
@@ -3758,12 +3769,12 @@
           <t>WACC privado (referencia)</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
-      <c r="E19" s="18" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>SWITCHING VALUE (USD/tCO2e)</t>
         </is>
@@ -3771,7 +3782,7 @@
       <c r="C21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="25" t="inlineStr">
         <is>
           <t>→ "Este proyecto se justifica socialmente si el carbono supera USD ___/tCO2e"</t>
         </is>

</xml_diff>